<commit_message>
Sensitivity-grondprijs-as genereren uit richtprijs-cel (C14) i.p.v. hardcoded
Data-only wijziging in Layers-Development-Plan-Hoofddorp-II-XL_leeg.xlsx:
de sensitivity-rijen (was B82:B86) berekenen nu C14*0.7..C14*1.3 in plaats
van vaste bedragen, zodat de as automatisch meeschaalt met de richtprijs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZo676XCJGcFYLkTMD4KwH
</commit_message>
<xml_diff>
--- a/Layers-Development-Plan-Hoofddorp-II-XL_leeg.xlsx
+++ b/Layers-Development-Plan-Hoofddorp-II-XL_leeg.xlsx
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="C53" s="75">
-        <f>IF(C49&lt;=C28,"PAST ✓","PAST NIET ✗ — meer lagen of minder BVO")</f>
+        <f>IF(C38=0,"—",IF(C49&lt;=C28,"PAST ✓","PAST NIET ✗ — meer lagen of minder BVO"))</f>
         <v/>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="C68" s="100">
-        <f>G38-C63</f>
+        <f>IF(C38=0,"—",G38-C63)</f>
         <v/>
       </c>
     </row>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C70" s="96">
-        <f>C68/C63</f>
+        <f>IF(C38=0,"—",IFERROR((G38-C63)/C63,""))</f>
         <v/>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="C76" s="101">
-        <f>G38-C75-C24*G38</f>
+        <f>IF(C38=0,"—",G38-C75-C24*G38)</f>
         <v/>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="C78" s="100">
-        <f>C76-C14</f>
+        <f>IF(C38=0,"—",C76-C14)</f>
         <v/>
       </c>
       <c r="E78" s="63" t="inlineStr">
@@ -1972,8 +1972,9 @@
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="60">
-      <c r="B82" s="104" t="n">
-        <v>3000000</v>
+      <c r="B82" s="104">
+        <f>C14*0.7</f>
+        <v/>
       </c>
       <c r="C82" s="105">
         <f>IFERROR(((G38*C81) - (B82+C58+C59+C61+C62+G38*C81*C21))/(G38*C81),"")</f>
@@ -1993,8 +1994,9 @@
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="60">
-      <c r="B83" s="104" t="n">
-        <v>3500000</v>
+      <c r="B83" s="104">
+        <f>C14*0.85</f>
+        <v/>
       </c>
       <c r="C83" s="105">
         <f>IFERROR(((G38*C81) - (B83+C58+C59+C61+C62+G38*C81*C21))/(G38*C81),"")</f>
@@ -2014,8 +2016,9 @@
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="60">
-      <c r="B84" s="104" t="n">
-        <v>4000000</v>
+      <c r="B84" s="104">
+        <f>C14</f>
+        <v/>
       </c>
       <c r="C84" s="105">
         <f>IFERROR(((G38*C81) - (B84+C58+C59+C61+C62+G38*C81*C21))/(G38*C81),"")</f>
@@ -2035,8 +2038,9 @@
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="60">
-      <c r="B85" s="104" t="n">
-        <v>4500000</v>
+      <c r="B85" s="104">
+        <f>C14*1.15</f>
+        <v/>
       </c>
       <c r="C85" s="105">
         <f>IFERROR(((G38*C81) - (B85+C58+C59+C61+C62+G38*C81*C21))/(G38*C81),"")</f>
@@ -2056,8 +2060,9 @@
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="60">
-      <c r="B86" s="104" t="n">
-        <v>5000000</v>
+      <c r="B86" s="104">
+        <f>C14*1.3</f>
+        <v/>
       </c>
       <c r="C86" s="105">
         <f>IFERROR(((G38*C81) - (B86+C58+C59+C61+C62+G38*C81*C21))/(G38*C81),"")</f>
@@ -2103,7 +2108,7 @@
         </is>
       </c>
       <c r="C90" s="109">
-        <f>C43</f>
+        <f>IF(C38=0,"—",C43)</f>
         <v/>
       </c>
       <c r="D90" s="110" t="inlineStr">
@@ -2196,7 +2201,7 @@
         </is>
       </c>
       <c r="C95" s="109">
-        <f>C48</f>
+        <f>IF(C38=0,"—",C48)</f>
         <v/>
       </c>
       <c r="D95" s="111" t="n"/>
@@ -2212,7 +2217,7 @@
         </is>
       </c>
       <c r="C96" s="109">
-        <f>E38</f>
+        <f>IF(C38=0,"—",E38)</f>
         <v/>
       </c>
       <c r="D96" s="111" t="n"/>
@@ -2228,7 +2233,7 @@
         </is>
       </c>
       <c r="C97" s="116">
-        <f>C38</f>
+        <f>IF(C38=0,"—",C38)</f>
         <v/>
       </c>
       <c r="D97" s="111" t="n"/>
@@ -2244,7 +2249,7 @@
         </is>
       </c>
       <c r="C98" s="114">
-        <f>F38</f>
+        <f>IF(C38=0,"—",F38)</f>
         <v/>
       </c>
       <c r="D98" s="110" t="inlineStr">
@@ -2264,7 +2269,7 @@
         </is>
       </c>
       <c r="C99" s="114">
-        <f>G38</f>
+        <f>IF(C38=0,"—",G38)</f>
         <v/>
       </c>
       <c r="D99" s="111" t="n"/>
@@ -2280,7 +2285,7 @@
         </is>
       </c>
       <c r="C100" s="114">
-        <f>C58</f>
+        <f>IF(C38=0,"—",C58)</f>
         <v/>
       </c>
       <c r="D100" s="111" t="n"/>
@@ -2296,7 +2301,7 @@
         </is>
       </c>
       <c r="C101" s="117">
-        <f>C54</f>
+        <f>IF(C38=0,"—",C54)</f>
         <v/>
       </c>
       <c r="D101" s="111" t="n"/>

</xml_diff>